<commit_message>
update gemini 2.5 pro flash
</commit_message>
<xml_diff>
--- a/test_results/gemini-2.5-pro/统计表格.xlsx
+++ b/test_results/gemini-2.5-pro/统计表格.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\111\新建文件夹\数据分析\分析结果\gemini-2.5-pro测试结果\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\111\LLM-NeedleInAHaystack\test_results\gemini-2.5-pro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A0212BF-08A1-49B7-B1E4-D42AC544A0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74D27CF5-542D-46A3-9BF9-F8D7A75C3333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{58898F7C-67C2-4EC0-A511-F699C1A6044A}"/>
+    <workbookView xWindow="1300" yWindow="360" windowWidth="21200" windowHeight="13630" xr2:uid="{58898F7C-67C2-4EC0-A511-F699C1A6044A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,27 +39,21 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>上下文对数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>上下文k</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>准确率分数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>测试场次</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>不遵守格式场次</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>json失败几率</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -174,6 +168,28 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-4.6802827965435979E-2"/>
+                  <c:y val="-4.0791901012373469E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-B25B-407D-B08E-C03DFEA2C337}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -241,40 +257,40 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.3010299956639813</c:v>
+                  <c:v>1.301029996</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.4771212547196624</c:v>
+                  <c:v>1.4771212549999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.6989700043360187</c:v>
+                  <c:v>1.698970004</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.8450980400142569</c:v>
+                  <c:v>1.8450980400000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.9030899869919435</c:v>
+                  <c:v>1.903089987</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.954242509439325</c:v>
+                  <c:v>1.954242509</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.1760912590556813</c:v>
+                  <c:v>2.1760912590000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.3010299956639813</c:v>
+                  <c:v>2.301029996</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.4771212547196626</c:v>
+                  <c:v>2.4771212550000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.6989700043360187</c:v>
+                  <c:v>2.698970004</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9542425094393248</c:v>
+                  <c:v>2.9542425090000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -295,34 +311,34 @@
                   <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>96.3</c:v>
+                  <c:v>97.78</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>86.02</c:v>
+                  <c:v>95.11</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>60.67</c:v>
+                  <c:v>83.83</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>33.25</c:v>
+                  <c:v>57.03</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>21.43</c:v>
+                  <c:v>37.479999999999997</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>6.94</c:v>
+                  <c:v>18.8</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5.55</c:v>
+                  <c:v>12.02</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.7</c:v>
+                  <c:v>6.06</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.17</c:v>
+                  <c:v>6.79</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.92</c:v>
+                  <c:v>7.48</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -350,6 +366,7 @@
         <c:axId val="1033575312"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="0.5"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -764,40 +781,40 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.3010299956639813</c:v>
+                  <c:v>1.301029996</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.4771212547196624</c:v>
+                  <c:v>1.4771212549999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.6989700043360187</c:v>
+                  <c:v>1.698970004</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.8450980400142569</c:v>
+                  <c:v>1.8450980400000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.9030899869919435</c:v>
+                  <c:v>1.903089987</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.954242509439325</c:v>
+                  <c:v>1.954242509</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2.1760912590556813</c:v>
+                  <c:v>2.1760912590000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2.3010299956639813</c:v>
+                  <c:v>2.301029996</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.4771212547196626</c:v>
+                  <c:v>2.4771212550000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2.6989700043360187</c:v>
+                  <c:v>2.698970004</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.9542425094393248</c:v>
+                  <c:v>2.9542425090000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -830,22 +847,22 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.3478260869565216E-2</c:v>
+                  <c:v>4.3478260999999997E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.11764705882352941</c:v>
+                  <c:v>0.117647059</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.43478260869565216</c:v>
+                  <c:v>0.43478260899999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.43333333333333335</c:v>
+                  <c:v>0.43333333299999999</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.32142857142857145</c:v>
+                  <c:v>0.321428571</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1016,6 +1033,7 @@
         <c:axId val="1062214144"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1199,6 +1217,601 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>准确率分数</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.5527777777777776E-2"/>
+                  <c:y val="-6.6804918101814825E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-C404-4004-A903-07B9DBE6EA3F}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.1638888888888888E-2"/>
+                  <c:y val="3.4799359973051495E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-AF4A-42C0-B74F-240CD243119E}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="zh-CN"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$7:$N$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>900</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$B$8:$N$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>97.78</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>95.11</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>83.83</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>57.03</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>37.479999999999997</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>18.8</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>12.02</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>6.06</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>6.79</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>7.48</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5801-404F-B2AA-4AA712860934}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="t"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="633438080"/>
+        <c:axId val="633438560"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="633438080"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>上下文长度</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" altLang="zh-CN" sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>/1000</a:t>
+                </a:r>
+                <a:endParaRPr lang="zh-CN" altLang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="zh-CN" altLang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="633438560"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="633438560"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>平均准确率得分</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" altLang="zh-CN" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                </a:endParaRPr>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US" altLang="zh-CN"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="633438080"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1279,6 +1892,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1796,6 +2449,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2318,13 +3487,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>139700</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>41274</xdr:rowOff>
+      <xdr:rowOff>41275</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>127000</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>19049</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2352,15 +3521,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>234950</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>120650</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>177799</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>184150</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>133349</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2380,6 +3549,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>215900</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>44450</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="图表 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C991328-BF01-6A21-A8F0-74D0C2C4BB08}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2708,7 +3913,7 @@
   <dimension ref="A6:N11"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.08203125" customWidth="1"/>
+    <col min="1" max="2" width="15.08203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -2716,56 +3921,43 @@
         <v>0</v>
       </c>
       <c r="B6">
-        <f>LOG10(B7)</f>
         <v>1</v>
       </c>
       <c r="C6">
-        <f>LOG10(C7)</f>
-        <v>1.3010299956639813</v>
+        <v>1.301029996</v>
       </c>
       <c r="D6">
-        <f>LOG10(D7)</f>
-        <v>1.4771212547196624</v>
+        <v>1.4771212549999999</v>
       </c>
       <c r="E6">
-        <f t="shared" ref="E6:N6" si="0">LOG10(E7)</f>
-        <v>1.6989700043360187</v>
+        <v>1.698970004</v>
       </c>
       <c r="F6">
-        <f t="shared" si="0"/>
-        <v>1.8450980400142569</v>
+        <v>1.8450980400000001</v>
       </c>
       <c r="G6">
-        <f t="shared" si="0"/>
-        <v>1.9030899869919435</v>
+        <v>1.903089987</v>
       </c>
       <c r="H6">
-        <f t="shared" si="0"/>
-        <v>1.954242509439325</v>
+        <v>1.954242509</v>
       </c>
       <c r="I6">
-        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="J6">
-        <f t="shared" si="0"/>
-        <v>2.1760912590556813</v>
+        <v>2.1760912590000001</v>
       </c>
       <c r="K6">
-        <f t="shared" si="0"/>
-        <v>2.3010299956639813</v>
+        <v>2.301029996</v>
       </c>
       <c r="L6">
-        <f t="shared" si="0"/>
-        <v>2.4771212547196626</v>
+        <v>2.4771212550000001</v>
       </c>
       <c r="M6">
-        <f t="shared" si="0"/>
-        <v>2.6989700043360187</v>
+        <v>2.698970004</v>
       </c>
       <c r="N6">
-        <f t="shared" si="0"/>
-        <v>2.9542425094393248</v>
+        <v>2.9542425090000002</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -2826,34 +4018,34 @@
         <v>100</v>
       </c>
       <c r="E8">
-        <v>96.3</v>
+        <v>97.78</v>
       </c>
       <c r="F8">
-        <v>86.02</v>
+        <v>95.11</v>
       </c>
       <c r="G8">
-        <v>60.67</v>
+        <v>83.83</v>
       </c>
       <c r="H8">
-        <v>33.25</v>
+        <v>57.03</v>
       </c>
       <c r="I8">
-        <v>21.43</v>
+        <v>37.479999999999997</v>
       </c>
       <c r="J8">
-        <v>6.94</v>
+        <v>18.8</v>
       </c>
       <c r="K8">
-        <v>5.55</v>
+        <v>12.02</v>
       </c>
       <c r="L8">
-        <v>2.7</v>
+        <v>6.06</v>
       </c>
       <c r="M8">
-        <v>2.17</v>
+        <v>6.79</v>
       </c>
       <c r="N8">
-        <v>1.92</v>
+        <v>7.48</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -2949,56 +4141,43 @@
         <v>5</v>
       </c>
       <c r="B11">
-        <f>B10/B9</f>
         <v>0</v>
       </c>
       <c r="C11">
-        <f t="shared" ref="C11:N11" si="1">C10/C9</f>
         <v>0</v>
       </c>
       <c r="D11">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="E11">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="F11">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G11">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H11">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="I11">
-        <f t="shared" si="1"/>
-        <v>4.3478260869565216E-2</v>
+        <v>4.3478260999999997E-2</v>
       </c>
       <c r="J11">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K11">
-        <f t="shared" si="1"/>
-        <v>0.11764705882352941</v>
+        <v>0.117647059</v>
       </c>
       <c r="L11">
-        <f t="shared" si="1"/>
-        <v>0.43478260869565216</v>
+        <v>0.43478260899999999</v>
       </c>
       <c r="M11">
-        <f t="shared" si="1"/>
-        <v>0.43333333333333335</v>
+        <v>0.43333333299999999</v>
       </c>
       <c r="N11">
-        <f t="shared" si="1"/>
-        <v>0.32142857142857145</v>
+        <v>0.321428571</v>
       </c>
     </row>
   </sheetData>

</xml_diff>